<commit_message>
fix: bereinige und härte Inseratsdatenflüsse
</commit_message>
<xml_diff>
--- a/public/Fabian-Pascal-Adressimport-Vorlage.xlsx
+++ b/public/Fabian-Pascal-Adressimport-Vorlage.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adressimport" sheetId="1" r:id="Red73f7f0c46c4b9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adressimport" sheetId="1" r:id="R0328cbed05a34f4c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -621,9 +621,7 @@
       <x:c r="N4" s="17" t="str">
         <x:v>Natur &amp; Freizeit</x:v>
       </x:c>
-      <x:c r="O4" s="18" t="str">
-        <x:v>Hinweise</x:v>
-      </x:c>
+      <x:c r="O4"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="30" t="str">
@@ -666,9 +664,7 @@
       <x:c r="N5" s="48" t="str">
         <x:v>Bestätigte Freizeit- und Naturangaben</x:v>
       </x:c>
-      <x:c r="O5" s="49" t="str">
-        <x:v>Beispielzeile vor dem eigenen Import löschen oder überschreiben</x:v>
-      </x:c>
+      <x:c r="O5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="33"/>
@@ -685,7 +681,7 @@
       <x:c r="L6" s="50"/>
       <x:c r="M6" s="50"/>
       <x:c r="N6" s="50"/>
-      <x:c r="O6" s="51"/>
+      <x:c r="O6"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="33"/>
@@ -702,7 +698,7 @@
       <x:c r="L7" s="50"/>
       <x:c r="M7" s="50"/>
       <x:c r="N7" s="50"/>
-      <x:c r="O7" s="51"/>
+      <x:c r="O7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="33"/>
@@ -719,7 +715,7 @@
       <x:c r="L8" s="50"/>
       <x:c r="M8" s="50"/>
       <x:c r="N8" s="50"/>
-      <x:c r="O8" s="51"/>
+      <x:c r="O8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="33"/>
@@ -736,7 +732,7 @@
       <x:c r="L9" s="50"/>
       <x:c r="M9" s="50"/>
       <x:c r="N9" s="50"/>
-      <x:c r="O9" s="51"/>
+      <x:c r="O9"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="33"/>
@@ -753,7 +749,7 @@
       <x:c r="L10" s="50"/>
       <x:c r="M10" s="50"/>
       <x:c r="N10" s="50"/>
-      <x:c r="O10" s="51"/>
+      <x:c r="O10"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="33"/>
@@ -770,7 +766,7 @@
       <x:c r="L11" s="50"/>
       <x:c r="M11" s="50"/>
       <x:c r="N11" s="50"/>
-      <x:c r="O11" s="51"/>
+      <x:c r="O11"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="33"/>
@@ -787,7 +783,7 @@
       <x:c r="L12" s="50"/>
       <x:c r="M12" s="50"/>
       <x:c r="N12" s="50"/>
-      <x:c r="O12" s="51"/>
+      <x:c r="O12"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="33"/>
@@ -804,7 +800,7 @@
       <x:c r="L13" s="50"/>
       <x:c r="M13" s="50"/>
       <x:c r="N13" s="50"/>
-      <x:c r="O13" s="51"/>
+      <x:c r="O13"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="33"/>
@@ -821,7 +817,7 @@
       <x:c r="L14" s="50"/>
       <x:c r="M14" s="50"/>
       <x:c r="N14" s="50"/>
-      <x:c r="O14" s="51"/>
+      <x:c r="O14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="33"/>
@@ -838,7 +834,7 @@
       <x:c r="L15" s="50"/>
       <x:c r="M15" s="50"/>
       <x:c r="N15" s="50"/>
-      <x:c r="O15" s="51"/>
+      <x:c r="O15"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="33"/>
@@ -855,7 +851,7 @@
       <x:c r="L16" s="50"/>
       <x:c r="M16" s="50"/>
       <x:c r="N16" s="50"/>
-      <x:c r="O16" s="51"/>
+      <x:c r="O16"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="33"/>
@@ -872,7 +868,7 @@
       <x:c r="L17" s="50"/>
       <x:c r="M17" s="50"/>
       <x:c r="N17" s="50"/>
-      <x:c r="O17" s="51"/>
+      <x:c r="O17"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="33"/>
@@ -889,7 +885,7 @@
       <x:c r="L18" s="50"/>
       <x:c r="M18" s="50"/>
       <x:c r="N18" s="50"/>
-      <x:c r="O18" s="51"/>
+      <x:c r="O18"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="33"/>
@@ -906,7 +902,7 @@
       <x:c r="L19" s="50"/>
       <x:c r="M19" s="50"/>
       <x:c r="N19" s="50"/>
-      <x:c r="O19" s="51"/>
+      <x:c r="O19"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="33"/>
@@ -923,7 +919,7 @@
       <x:c r="L20" s="50"/>
       <x:c r="M20" s="50"/>
       <x:c r="N20" s="50"/>
-      <x:c r="O20" s="51"/>
+      <x:c r="O20"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="33"/>
@@ -940,7 +936,7 @@
       <x:c r="L21" s="50"/>
       <x:c r="M21" s="50"/>
       <x:c r="N21" s="50"/>
-      <x:c r="O21" s="51"/>
+      <x:c r="O21"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="33"/>
@@ -957,7 +953,7 @@
       <x:c r="L22" s="50"/>
       <x:c r="M22" s="50"/>
       <x:c r="N22" s="50"/>
-      <x:c r="O22" s="51"/>
+      <x:c r="O22"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="33"/>
@@ -974,7 +970,7 @@
       <x:c r="L23" s="50"/>
       <x:c r="M23" s="50"/>
       <x:c r="N23" s="50"/>
-      <x:c r="O23" s="51"/>
+      <x:c r="O23"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="33"/>
@@ -991,7 +987,7 @@
       <x:c r="L24" s="50"/>
       <x:c r="M24" s="50"/>
       <x:c r="N24" s="50"/>
-      <x:c r="O24" s="51"/>
+      <x:c r="O24"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="33"/>
@@ -1008,7 +1004,7 @@
       <x:c r="L25" s="50"/>
       <x:c r="M25" s="50"/>
       <x:c r="N25" s="50"/>
-      <x:c r="O25" s="51"/>
+      <x:c r="O25"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="33"/>
@@ -1025,7 +1021,7 @@
       <x:c r="L26" s="50"/>
       <x:c r="M26" s="50"/>
       <x:c r="N26" s="50"/>
-      <x:c r="O26" s="51"/>
+      <x:c r="O26"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="33"/>
@@ -1042,7 +1038,7 @@
       <x:c r="L27" s="50"/>
       <x:c r="M27" s="50"/>
       <x:c r="N27" s="50"/>
-      <x:c r="O27" s="51"/>
+      <x:c r="O27"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="33"/>
@@ -1059,7 +1055,7 @@
       <x:c r="L28" s="50"/>
       <x:c r="M28" s="50"/>
       <x:c r="N28" s="50"/>
-      <x:c r="O28" s="51"/>
+      <x:c r="O28"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="33"/>
@@ -1076,7 +1072,7 @@
       <x:c r="L29" s="50"/>
       <x:c r="M29" s="50"/>
       <x:c r="N29" s="50"/>
-      <x:c r="O29" s="51"/>
+      <x:c r="O29"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="33"/>
@@ -1093,7 +1089,7 @@
       <x:c r="L30" s="50"/>
       <x:c r="M30" s="50"/>
       <x:c r="N30" s="50"/>
-      <x:c r="O30" s="51"/>
+      <x:c r="O30"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="33"/>
@@ -1110,7 +1106,7 @@
       <x:c r="L31" s="50"/>
       <x:c r="M31" s="50"/>
       <x:c r="N31" s="50"/>
-      <x:c r="O31" s="51"/>
+      <x:c r="O31"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="33"/>
@@ -1127,7 +1123,7 @@
       <x:c r="L32" s="50"/>
       <x:c r="M32" s="50"/>
       <x:c r="N32" s="50"/>
-      <x:c r="O32" s="51"/>
+      <x:c r="O32"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="33"/>
@@ -1144,7 +1140,7 @@
       <x:c r="L33" s="50"/>
       <x:c r="M33" s="50"/>
       <x:c r="N33" s="50"/>
-      <x:c r="O33" s="51"/>
+      <x:c r="O33"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="33"/>
@@ -1161,7 +1157,7 @@
       <x:c r="L34" s="50"/>
       <x:c r="M34" s="50"/>
       <x:c r="N34" s="50"/>
-      <x:c r="O34" s="51"/>
+      <x:c r="O34"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="33"/>
@@ -1178,7 +1174,7 @@
       <x:c r="L35" s="50"/>
       <x:c r="M35" s="50"/>
       <x:c r="N35" s="50"/>
-      <x:c r="O35" s="51"/>
+      <x:c r="O35"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="33"/>
@@ -1195,7 +1191,7 @@
       <x:c r="L36" s="50"/>
       <x:c r="M36" s="50"/>
       <x:c r="N36" s="50"/>
-      <x:c r="O36" s="51"/>
+      <x:c r="O36"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="33"/>
@@ -1212,7 +1208,7 @@
       <x:c r="L37" s="50"/>
       <x:c r="M37" s="50"/>
       <x:c r="N37" s="50"/>
-      <x:c r="O37" s="51"/>
+      <x:c r="O37"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="33"/>
@@ -1229,7 +1225,7 @@
       <x:c r="L38" s="50"/>
       <x:c r="M38" s="50"/>
       <x:c r="N38" s="50"/>
-      <x:c r="O38" s="51"/>
+      <x:c r="O38"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="33"/>
@@ -1246,7 +1242,7 @@
       <x:c r="L39" s="50"/>
       <x:c r="M39" s="50"/>
       <x:c r="N39" s="50"/>
-      <x:c r="O39" s="51"/>
+      <x:c r="O39"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="33"/>
@@ -1263,7 +1259,7 @@
       <x:c r="L40" s="50"/>
       <x:c r="M40" s="50"/>
       <x:c r="N40" s="50"/>
-      <x:c r="O40" s="51"/>
+      <x:c r="O40"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="33"/>
@@ -1280,7 +1276,7 @@
       <x:c r="L41" s="50"/>
       <x:c r="M41" s="50"/>
       <x:c r="N41" s="50"/>
-      <x:c r="O41" s="51"/>
+      <x:c r="O41"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="33"/>
@@ -1297,7 +1293,7 @@
       <x:c r="L42" s="50"/>
       <x:c r="M42" s="50"/>
       <x:c r="N42" s="50"/>
-      <x:c r="O42" s="51"/>
+      <x:c r="O42"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="33"/>
@@ -1314,7 +1310,7 @@
       <x:c r="L43" s="50"/>
       <x:c r="M43" s="50"/>
       <x:c r="N43" s="50"/>
-      <x:c r="O43" s="51"/>
+      <x:c r="O43"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="33"/>
@@ -1331,7 +1327,7 @@
       <x:c r="L44" s="50"/>
       <x:c r="M44" s="50"/>
       <x:c r="N44" s="50"/>
-      <x:c r="O44" s="51"/>
+      <x:c r="O44"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="33"/>
@@ -1348,7 +1344,7 @@
       <x:c r="L45" s="50"/>
       <x:c r="M45" s="50"/>
       <x:c r="N45" s="50"/>
-      <x:c r="O45" s="51"/>
+      <x:c r="O45"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="33"/>
@@ -1365,7 +1361,7 @@
       <x:c r="L46" s="50"/>
       <x:c r="M46" s="50"/>
       <x:c r="N46" s="50"/>
-      <x:c r="O46" s="51"/>
+      <x:c r="O46"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="33"/>
@@ -1382,7 +1378,7 @@
       <x:c r="L47" s="50"/>
       <x:c r="M47" s="50"/>
       <x:c r="N47" s="50"/>
-      <x:c r="O47" s="51"/>
+      <x:c r="O47"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="33"/>
@@ -1399,7 +1395,7 @@
       <x:c r="L48" s="50"/>
       <x:c r="M48" s="50"/>
       <x:c r="N48" s="50"/>
-      <x:c r="O48" s="51"/>
+      <x:c r="O48"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="33"/>
@@ -1416,7 +1412,7 @@
       <x:c r="L49" s="50"/>
       <x:c r="M49" s="50"/>
       <x:c r="N49" s="50"/>
-      <x:c r="O49" s="51"/>
+      <x:c r="O49"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="33"/>
@@ -1433,7 +1429,7 @@
       <x:c r="L50" s="50"/>
       <x:c r="M50" s="50"/>
       <x:c r="N50" s="50"/>
-      <x:c r="O50" s="51"/>
+      <x:c r="O50"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="33"/>
@@ -1450,7 +1446,7 @@
       <x:c r="L51" s="50"/>
       <x:c r="M51" s="50"/>
       <x:c r="N51" s="50"/>
-      <x:c r="O51" s="51"/>
+      <x:c r="O51"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="33"/>
@@ -1467,7 +1463,7 @@
       <x:c r="L52" s="50"/>
       <x:c r="M52" s="50"/>
       <x:c r="N52" s="50"/>
-      <x:c r="O52" s="51"/>
+      <x:c r="O52"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="33"/>
@@ -1484,7 +1480,7 @@
       <x:c r="L53" s="50"/>
       <x:c r="M53" s="50"/>
       <x:c r="N53" s="50"/>
-      <x:c r="O53" s="51"/>
+      <x:c r="O53"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="33"/>
@@ -1501,7 +1497,7 @@
       <x:c r="L54" s="50"/>
       <x:c r="M54" s="50"/>
       <x:c r="N54" s="50"/>
-      <x:c r="O54" s="51"/>
+      <x:c r="O54"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="33"/>
@@ -1518,7 +1514,7 @@
       <x:c r="L55" s="50"/>
       <x:c r="M55" s="50"/>
       <x:c r="N55" s="50"/>
-      <x:c r="O55" s="51"/>
+      <x:c r="O55"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="33"/>
@@ -1535,7 +1531,7 @@
       <x:c r="L56" s="50"/>
       <x:c r="M56" s="50"/>
       <x:c r="N56" s="50"/>
-      <x:c r="O56" s="51"/>
+      <x:c r="O56"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="33"/>
@@ -1552,7 +1548,7 @@
       <x:c r="L57" s="50"/>
       <x:c r="M57" s="50"/>
       <x:c r="N57" s="50"/>
-      <x:c r="O57" s="51"/>
+      <x:c r="O57"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="33"/>
@@ -1569,7 +1565,7 @@
       <x:c r="L58" s="50"/>
       <x:c r="M58" s="50"/>
       <x:c r="N58" s="50"/>
-      <x:c r="O58" s="51"/>
+      <x:c r="O58"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="33"/>
@@ -1586,7 +1582,7 @@
       <x:c r="L59" s="50"/>
       <x:c r="M59" s="50"/>
       <x:c r="N59" s="50"/>
-      <x:c r="O59" s="51"/>
+      <x:c r="O59"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="33"/>
@@ -1603,7 +1599,7 @@
       <x:c r="L60" s="50"/>
       <x:c r="M60" s="50"/>
       <x:c r="N60" s="50"/>
-      <x:c r="O60" s="51"/>
+      <x:c r="O60"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="33"/>
@@ -1620,7 +1616,7 @@
       <x:c r="L61" s="50"/>
       <x:c r="M61" s="50"/>
       <x:c r="N61" s="50"/>
-      <x:c r="O61" s="51"/>
+      <x:c r="O61"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="33"/>
@@ -1637,7 +1633,7 @@
       <x:c r="L62" s="50"/>
       <x:c r="M62" s="50"/>
       <x:c r="N62" s="50"/>
-      <x:c r="O62" s="51"/>
+      <x:c r="O62"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="33"/>
@@ -1654,7 +1650,7 @@
       <x:c r="L63" s="50"/>
       <x:c r="M63" s="50"/>
       <x:c r="N63" s="50"/>
-      <x:c r="O63" s="51"/>
+      <x:c r="O63"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="33"/>
@@ -1671,7 +1667,7 @@
       <x:c r="L64" s="50"/>
       <x:c r="M64" s="50"/>
       <x:c r="N64" s="50"/>
-      <x:c r="O64" s="51"/>
+      <x:c r="O64"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="33"/>
@@ -1688,7 +1684,7 @@
       <x:c r="L65" s="50"/>
       <x:c r="M65" s="50"/>
       <x:c r="N65" s="50"/>
-      <x:c r="O65" s="51"/>
+      <x:c r="O65"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="33"/>
@@ -1705,7 +1701,7 @@
       <x:c r="L66" s="50"/>
       <x:c r="M66" s="50"/>
       <x:c r="N66" s="50"/>
-      <x:c r="O66" s="51"/>
+      <x:c r="O66"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="33"/>
@@ -1722,7 +1718,7 @@
       <x:c r="L67" s="50"/>
       <x:c r="M67" s="50"/>
       <x:c r="N67" s="50"/>
-      <x:c r="O67" s="51"/>
+      <x:c r="O67"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="33"/>
@@ -1739,7 +1735,7 @@
       <x:c r="L68" s="50"/>
       <x:c r="M68" s="50"/>
       <x:c r="N68" s="50"/>
-      <x:c r="O68" s="51"/>
+      <x:c r="O68"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="33"/>
@@ -1756,7 +1752,7 @@
       <x:c r="L69" s="50"/>
       <x:c r="M69" s="50"/>
       <x:c r="N69" s="50"/>
-      <x:c r="O69" s="51"/>
+      <x:c r="O69"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="33"/>
@@ -1773,7 +1769,7 @@
       <x:c r="L70" s="50"/>
       <x:c r="M70" s="50"/>
       <x:c r="N70" s="50"/>
-      <x:c r="O70" s="51"/>
+      <x:c r="O70"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="33"/>
@@ -1790,7 +1786,7 @@
       <x:c r="L71" s="50"/>
       <x:c r="M71" s="50"/>
       <x:c r="N71" s="50"/>
-      <x:c r="O71" s="51"/>
+      <x:c r="O71"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="33"/>
@@ -1807,7 +1803,7 @@
       <x:c r="L72" s="50"/>
       <x:c r="M72" s="50"/>
       <x:c r="N72" s="50"/>
-      <x:c r="O72" s="51"/>
+      <x:c r="O72"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="33"/>
@@ -1824,7 +1820,7 @@
       <x:c r="L73" s="50"/>
       <x:c r="M73" s="50"/>
       <x:c r="N73" s="50"/>
-      <x:c r="O73" s="51"/>
+      <x:c r="O73"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="33"/>
@@ -1841,7 +1837,7 @@
       <x:c r="L74" s="50"/>
       <x:c r="M74" s="50"/>
       <x:c r="N74" s="50"/>
-      <x:c r="O74" s="51"/>
+      <x:c r="O74"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="33"/>
@@ -1858,7 +1854,7 @@
       <x:c r="L75" s="50"/>
       <x:c r="M75" s="50"/>
       <x:c r="N75" s="50"/>
-      <x:c r="O75" s="51"/>
+      <x:c r="O75"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="33"/>
@@ -1875,7 +1871,7 @@
       <x:c r="L76" s="50"/>
       <x:c r="M76" s="50"/>
       <x:c r="N76" s="50"/>
-      <x:c r="O76" s="51"/>
+      <x:c r="O76"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="33"/>
@@ -1892,7 +1888,7 @@
       <x:c r="L77" s="50"/>
       <x:c r="M77" s="50"/>
       <x:c r="N77" s="50"/>
-      <x:c r="O77" s="51"/>
+      <x:c r="O77"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="33"/>
@@ -1909,7 +1905,7 @@
       <x:c r="L78" s="50"/>
       <x:c r="M78" s="50"/>
       <x:c r="N78" s="50"/>
-      <x:c r="O78" s="51"/>
+      <x:c r="O78"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="33"/>
@@ -1926,7 +1922,7 @@
       <x:c r="L79" s="50"/>
       <x:c r="M79" s="50"/>
       <x:c r="N79" s="50"/>
-      <x:c r="O79" s="51"/>
+      <x:c r="O79"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="33"/>
@@ -1943,7 +1939,7 @@
       <x:c r="L80" s="50"/>
       <x:c r="M80" s="50"/>
       <x:c r="N80" s="50"/>
-      <x:c r="O80" s="51"/>
+      <x:c r="O80"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="33"/>
@@ -1960,7 +1956,7 @@
       <x:c r="L81" s="50"/>
       <x:c r="M81" s="50"/>
       <x:c r="N81" s="50"/>
-      <x:c r="O81" s="51"/>
+      <x:c r="O81"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="33"/>
@@ -1977,7 +1973,7 @@
       <x:c r="L82" s="50"/>
       <x:c r="M82" s="50"/>
       <x:c r="N82" s="50"/>
-      <x:c r="O82" s="51"/>
+      <x:c r="O82"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="33"/>
@@ -1994,7 +1990,7 @@
       <x:c r="L83" s="50"/>
       <x:c r="M83" s="50"/>
       <x:c r="N83" s="50"/>
-      <x:c r="O83" s="51"/>
+      <x:c r="O83"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="33"/>
@@ -2011,7 +2007,7 @@
       <x:c r="L84" s="50"/>
       <x:c r="M84" s="50"/>
       <x:c r="N84" s="50"/>
-      <x:c r="O84" s="51"/>
+      <x:c r="O84"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="33"/>
@@ -2028,7 +2024,7 @@
       <x:c r="L85" s="50"/>
       <x:c r="M85" s="50"/>
       <x:c r="N85" s="50"/>
-      <x:c r="O85" s="51"/>
+      <x:c r="O85"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="33"/>
@@ -2045,7 +2041,7 @@
       <x:c r="L86" s="50"/>
       <x:c r="M86" s="50"/>
       <x:c r="N86" s="50"/>
-      <x:c r="O86" s="51"/>
+      <x:c r="O86"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="33"/>
@@ -2062,7 +2058,7 @@
       <x:c r="L87" s="50"/>
       <x:c r="M87" s="50"/>
       <x:c r="N87" s="50"/>
-      <x:c r="O87" s="51"/>
+      <x:c r="O87"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="33"/>
@@ -2079,7 +2075,7 @@
       <x:c r="L88" s="50"/>
       <x:c r="M88" s="50"/>
       <x:c r="N88" s="50"/>
-      <x:c r="O88" s="51"/>
+      <x:c r="O88"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="33"/>
@@ -2096,7 +2092,7 @@
       <x:c r="L89" s="50"/>
       <x:c r="M89" s="50"/>
       <x:c r="N89" s="50"/>
-      <x:c r="O89" s="51"/>
+      <x:c r="O89"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="33"/>
@@ -2113,7 +2109,7 @@
       <x:c r="L90" s="50"/>
       <x:c r="M90" s="50"/>
       <x:c r="N90" s="50"/>
-      <x:c r="O90" s="51"/>
+      <x:c r="O90"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="33"/>
@@ -2130,7 +2126,7 @@
       <x:c r="L91" s="50"/>
       <x:c r="M91" s="50"/>
       <x:c r="N91" s="50"/>
-      <x:c r="O91" s="51"/>
+      <x:c r="O91"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="33"/>
@@ -2147,7 +2143,7 @@
       <x:c r="L92" s="50"/>
       <x:c r="M92" s="50"/>
       <x:c r="N92" s="50"/>
-      <x:c r="O92" s="51"/>
+      <x:c r="O92"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="33"/>
@@ -2164,7 +2160,7 @@
       <x:c r="L93" s="50"/>
       <x:c r="M93" s="50"/>
       <x:c r="N93" s="50"/>
-      <x:c r="O93" s="51"/>
+      <x:c r="O93"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="33"/>
@@ -2181,7 +2177,7 @@
       <x:c r="L94" s="50"/>
       <x:c r="M94" s="50"/>
       <x:c r="N94" s="50"/>
-      <x:c r="O94" s="51"/>
+      <x:c r="O94"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="33"/>
@@ -2198,7 +2194,7 @@
       <x:c r="L95" s="50"/>
       <x:c r="M95" s="50"/>
       <x:c r="N95" s="50"/>
-      <x:c r="O95" s="51"/>
+      <x:c r="O95"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="33"/>
@@ -2215,7 +2211,7 @@
       <x:c r="L96" s="50"/>
       <x:c r="M96" s="50"/>
       <x:c r="N96" s="50"/>
-      <x:c r="O96" s="51"/>
+      <x:c r="O96"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="33"/>
@@ -2232,7 +2228,7 @@
       <x:c r="L97" s="50"/>
       <x:c r="M97" s="50"/>
       <x:c r="N97" s="50"/>
-      <x:c r="O97" s="51"/>
+      <x:c r="O97"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="33"/>
@@ -2249,7 +2245,7 @@
       <x:c r="L98" s="50"/>
       <x:c r="M98" s="50"/>
       <x:c r="N98" s="50"/>
-      <x:c r="O98" s="51"/>
+      <x:c r="O98"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="33"/>
@@ -2266,7 +2262,7 @@
       <x:c r="L99" s="50"/>
       <x:c r="M99" s="50"/>
       <x:c r="N99" s="50"/>
-      <x:c r="O99" s="51"/>
+      <x:c r="O99"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="33"/>
@@ -2283,7 +2279,7 @@
       <x:c r="L100" s="50"/>
       <x:c r="M100" s="50"/>
       <x:c r="N100" s="50"/>
-      <x:c r="O100" s="51"/>
+      <x:c r="O100"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="33"/>
@@ -2300,7 +2296,7 @@
       <x:c r="L101" s="50"/>
       <x:c r="M101" s="50"/>
       <x:c r="N101" s="50"/>
-      <x:c r="O101" s="51"/>
+      <x:c r="O101"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="33"/>
@@ -2317,7 +2313,7 @@
       <x:c r="L102" s="50"/>
       <x:c r="M102" s="50"/>
       <x:c r="N102" s="50"/>
-      <x:c r="O102" s="51"/>
+      <x:c r="O102"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="33"/>
@@ -2334,7 +2330,7 @@
       <x:c r="L103" s="50"/>
       <x:c r="M103" s="50"/>
       <x:c r="N103" s="50"/>
-      <x:c r="O103" s="51"/>
+      <x:c r="O103"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="36"/>
@@ -2351,7 +2347,7 @@
       <x:c r="L104" s="52"/>
       <x:c r="M104" s="52"/>
       <x:c r="N104" s="52"/>
-      <x:c r="O104" s="53"/>
+      <x:c r="O104"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>